<commit_message>
used function for date diff, end of month
</commit_message>
<xml_diff>
--- a/EXCEL/Date and Time Functions.xlsx
+++ b/EXCEL/Date and Time Functions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/898af4500e89e0da/Desktop/DHRUV/Data Science and Analytics with GenAl/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="8_{60DE7DFA-A72F-4513-A82F-32C35E916A33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1721C10-1D40-4BBE-881D-33C09FA5D6E6}"/>
+  <xr:revisionPtr revIDLastSave="40" documentId="8_{60DE7DFA-A72F-4513-A82F-32C35E916A33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F2AC2D3D-A766-4ED2-92A7-A91289FEE9A6}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{83374882-0478-4D90-A783-7BD1D4D12D8E}"/>
+    <workbookView minimized="1" xWindow="1776" yWindow="1776" windowWidth="17280" windowHeight="10500" xr2:uid="{83374882-0478-4D90-A783-7BD1D4D12D8E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>ID</t>
   </si>
@@ -75,6 +75,15 @@
   </si>
   <si>
     <t>day</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>date diff b/w join and end date</t>
+  </si>
+  <si>
+    <t>net working day</t>
   </si>
 </sst>
 </file>
@@ -465,7 +474,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A66E3EA-7351-4141-8EB0-580957AAF064}">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="5" max="5" width="9.92578125" bestFit="1" customWidth="1"/>
@@ -473,7 +482,7 @@
     <col min="9" max="9" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="63" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -498,8 +507,14 @@
       <c r="H1" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A2" s="2">
         <v>101</v>
       </c>
@@ -527,8 +542,16 @@
         <f>YEAR(C2)</f>
         <v>2022</v>
       </c>
+      <c r="I2">
+        <f>DATEDIF(C2,D2,"D")</f>
+        <v>1095</v>
+      </c>
+      <c r="J2">
+        <f>NETWORKDAYS(C2,D2)</f>
+        <v>782</v>
+      </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
         <v>102</v>
       </c>
@@ -556,8 +579,16 @@
         <f t="shared" ref="H3:H6" si="2">YEAR(C3)</f>
         <v>2021</v>
       </c>
+      <c r="I3">
+        <f t="shared" ref="I3:I6" si="3">DATEDIF(C3,D3,"D")</f>
+        <v>1461</v>
+      </c>
+      <c r="J3">
+        <f t="shared" ref="J3:J6" si="4">NETWORKDAYS(C3,D3)</f>
+        <v>1045</v>
+      </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
         <v>103</v>
       </c>
@@ -585,8 +616,16 @@
         <f t="shared" si="2"/>
         <v>2020</v>
       </c>
+      <c r="I4">
+        <f t="shared" si="3"/>
+        <v>1094</v>
+      </c>
+      <c r="J4">
+        <f t="shared" si="4"/>
+        <v>781</v>
+      </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>104</v>
       </c>
@@ -614,8 +653,16 @@
         <f t="shared" si="2"/>
         <v>2023</v>
       </c>
+      <c r="I5">
+        <f t="shared" si="3"/>
+        <v>1095</v>
+      </c>
+      <c r="J5">
+        <f t="shared" si="4"/>
+        <v>783</v>
+      </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A6" s="2">
         <v>105</v>
       </c>
@@ -643,16 +690,24 @@
         <f t="shared" si="2"/>
         <v>2022</v>
       </c>
+      <c r="I6">
+        <f t="shared" si="3"/>
+        <v>731</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="4"/>
+        <v>523</v>
+      </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.4">
-      <c r="E9" s="4">
-        <f ca="1">TODAY()</f>
-        <v>46251</v>
-      </c>
-      <c r="I9" s="5">
-        <f ca="1">NOW()</f>
-        <v>46251.977066782405</v>
-      </c>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="E9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I9" s="5"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.4">
+      <c r="E12" s="4"/>
+      <c r="I12" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add Lookups workbook and update Date and Time Functions
</commit_message>
<xml_diff>
--- a/EXCEL/Date and Time Functions.xlsx
+++ b/EXCEL/Date and Time Functions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/898af4500e89e0da/Desktop/DHRUV/Data Science and Analytics with GenAl/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="40" documentId="8_{60DE7DFA-A72F-4513-A82F-32C35E916A33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F2AC2D3D-A766-4ED2-92A7-A91289FEE9A6}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="8_{60DE7DFA-A72F-4513-A82F-32C35E916A33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F09C394-E7ED-4858-96BC-6D777D1F2380}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1776" yWindow="1776" windowWidth="17280" windowHeight="10500" xr2:uid="{83374882-0478-4D90-A783-7BD1D4D12D8E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{83374882-0478-4D90-A783-7BD1D4D12D8E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -478,7 +478,7 @@
   <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="5" max="5" width="9.92578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="8" width="0" hidden="1" customWidth="1"/>
+    <col min="6" max="8" width="9.140625" customWidth="1"/>
     <col min="9" max="9" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>